<commit_message>
docs(docs): registrar las decisiones D1 a D7 sobre las reglas abiertas
Escala de 1 a 100 sin 0, redondeo 0,5 hacia arriba, nota anual como promedio de los trimestres, dimensión sin notas
como pendiente, licencias como asistencia, riesgo con asistencia menor que 80 % y avisos en el sistema y por correo.
Se actualizan el Excel del backlog, el generador, las historias, el SRS y el ADR-0004.

Refs: T-004
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -266,7 +266,7 @@
     <t xml:space="preserve">BAJA</t>
   </si>
   <si>
-    <t xml:space="preserve">Depende de US-02 y US-06. Requiere definir el canal de notificación (propuesta: correo + aviso en el sistema).</t>
+    <t xml:space="preserve">Depende de US-02 y US-06. Canal de notificación: aviso en el sistema y correo (decisión D7 de `docs/backlog/reglas-ministerio.md`).</t>
   </si>
   <si>
     <t xml:space="preserve">US-12</t>
@@ -1094,7 +1094,7 @@
     <t xml:space="preserve">El pipeline está sano: lint, pruebas, cobertura, Quality Gate y auditoría de dependencias en verde.</t>
   </si>
   <si>
-    <t xml:space="preserve">Checks obligatorios del pull request</t>
+    <t xml:space="preserve">Build de Jenkins del commit en develop (ADR-0008)</t>
   </si>
   <si>
     <t xml:space="preserve">Cobertura ≥ 80 % en código nuevo y ≥ 90 % en el módulo de cálculo, exigida por la herramienta.</t>
@@ -1103,10 +1103,10 @@
     <t xml:space="preserve">coverageThreshold de Jest y Quality Gate</t>
   </si>
   <si>
-    <t xml:space="preserve">El pull request lo aprobó el otro integrante; nadie aprueba su propio código.</t>
+    <t xml:space="preserve">El otro integrante revisó sus commits en develop; nadie aprueba su propio código.</t>
   </si>
   <si>
-    <t xml:space="preserve">Historial del PR en GitHub</t>
+    <t xml:space="preserve">Comentarios de revisión en los commits de GitHub</t>
   </si>
   <si>
     <t xml:space="preserve">Está desplegada en staging y el smoke test pasa con el commit correcto.</t>
@@ -1196,7 +1196,7 @@
     <t xml:space="preserve">Dado un profesor en una materia asignada y un trimestre abierto, cuando registra la nota de una actividad dentro de una dimensión (Ser, Saber, Hacer o Autoevaluación) en la escala de 1 a 100, entonces la nota se guarda y aparece en la planilla.</t>
   </si>
   <si>
-    <t xml:space="preserve">❓ Dado un valor fuera de 1 a 100 [confirmar con el cliente si se admite 0 para actividades no presentadas], vacío o no numérico, cuando intenta guardar, entonces aparece un mensaje junto al campo y no se guarda nada.</t>
+    <t xml:space="preserve">Dado un valor fuera de 1 a 100 (no se admite 0; una actividad no presentada se registra con 1, decisión D1), vacío o no numérico, cuando intenta guardar, entonces aparece un mensaje junto al campo y no se guarda nada.</t>
   </si>
   <si>
     <t xml:space="preserve">M01</t>
@@ -1238,7 +1238,7 @@
     <t xml:space="preserve">RNF-01, R02</t>
   </si>
   <si>
-    <t xml:space="preserve">❓ Dado las notas de los tres trimestres, cuando se calcula la nota anual de la materia, entonces es el promedio de los tres trimestres redondeado al entero [confirmar con el texto del reglamento de evaluación vigente].</t>
+    <t xml:space="preserve">Dado las notas de los tres trimestres, cuando se calcula la nota anual de la materia, entonces es el promedio de los tres trimestres redondeado al entero, 0,5 hacia arriba (decisiones D2 y D3).</t>
   </si>
   <si>
     <t xml:space="preserve">Dado la tabla de casos de prueba firmada por el cliente (semilla en la hoja Reglas MinEdu), cuando corre la suite, entonces el 100 % de los casos da el resultado esperado.</t>
@@ -1247,7 +1247,7 @@
     <t xml:space="preserve">M01, R02</t>
   </si>
   <si>
-    <t xml:space="preserve">❓ Dado una dimensión que todavía no tiene actividades con nota, cuando se calcula la nota parcial del trimestre, entonces [definir con el cliente: se muestra como "pendiente" o cuenta como 0].</t>
+    <t xml:space="preserve">Dado una dimensión que todavía no tiene actividades con nota, cuando se calcula la nota parcial del trimestre, entonces la nota trimestral se muestra como "pendiente" e indica qué dimensiones faltan (decisión D4).</t>
   </si>
   <si>
     <t xml:space="preserve">Dado una nota registrada, cuando el profesor la corrige, entonces el sistema exige un motivo y guarda quién la cambió, la fecha y hora, el valor anterior y el nuevo.</t>
@@ -1268,7 +1268,7 @@
     <t xml:space="preserve">Dado una clase de su materia, cuando el profesor marca a cada estudiante como presente, ausente o con licencia, entonces se guarda la asistencia de esa fecha.</t>
   </si>
   <si>
-    <t xml:space="preserve">❓ Dado las asistencias registradas, cuando se calcula el porcentaje, entonces es (presentes [+ licencias, confirmar con el cliente]) / clases dictadas × 100, redondeado a un decimal.</t>
+    <t xml:space="preserve">Dado las asistencias registradas, cuando se calcula el porcentaje, entonces es (presentes + licencias) / clases dictadas × 100, redondeado a un decimal (decisión D5).</t>
   </si>
   <si>
     <t xml:space="preserve">Dado una fecha futura, cuando el profesor intenta registrar asistencia, entonces el sistema lo impide.</t>
@@ -1292,7 +1292,7 @@
     <t xml:space="preserve">Dado un curso del profesor, cuando abre el panel, entonces ve a cada estudiante con su promedio actual y su porcentaje de asistencia.</t>
   </si>
   <si>
-    <t xml:space="preserve">❓ Dado un estudiante con promedio menor que 51 o asistencia menor que [umbral a definir con el cliente, p. ej. 80 %], cuando se muestra el panel, entonces aparece marcado como "en riesgo".</t>
+    <t xml:space="preserve">Dado un estudiante con promedio menor que 51 o asistencia menor que 80 % (umbral configurable por gestión, decisión D6), cuando se muestra el panel, entonces aparece marcado como "en riesgo".</t>
   </si>
   <si>
     <t xml:space="preserve">Dado un estudiante, cuando el profesor genera su boletín, entonces el PDF muestra la unidad educativa, el código SIE, el nivel, el año de escolaridad y el paralelo, y por cada materia la nota de cada trimestre, la nota anual y el porcentaje de asistencia, iguales a los que muestra el sistema.</t>
@@ -1376,13 +1376,13 @@
     <t xml:space="preserve">Escala de calificación</t>
   </si>
   <si>
-    <t xml:space="preserve">1 a 100</t>
+    <t xml:space="preserve">1 a 100 (sin 0)</t>
   </si>
   <si>
     <t xml:space="preserve">Ministerio de Educación, vigente desde 2013</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmar si se admite 0</t>
+    <t xml:space="preserve">Decidido (D1)</t>
   </si>
   <si>
     <t xml:space="preserve">Nota mínima de aprobación</t>
@@ -1415,13 +1415,13 @@
     <t xml:space="preserve">Práctica habitual; no se encontró el texto oficial</t>
   </si>
   <si>
-    <t xml:space="preserve">❓ Confirmar con el reglamento completo</t>
+    <t xml:space="preserve">Decidido (D3)</t>
   </si>
   <si>
     <t xml:space="preserve">Suma de dimensiones (debe ser 100)</t>
   </si>
   <si>
-    <t xml:space="preserve">❓ Confirmar con el cliente</t>
+    <t xml:space="preserve">Confirmado</t>
   </si>
   <si>
     <t xml:space="preserve">Casos de ejemplo del cálculo (semilla de la tabla que firma el cliente, riesgo R02)</t>

</xml_diff>

<commit_message>
docs(docs): documentar el despliegue continuo desde el Sprint 1
ADR-0009: API y web en Render y despliegue continuo a staging desde el Sprint 1. T-028 y T-029 pasan al Sprint 1 en
el backlog. Guía de despliegue paso a paso; SAD, SRS y SQAP sin Vercel.

Refs: T-028
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -377,7 +377,7 @@
     <t xml:space="preserve">Semana 1. Un profesor inicia sesión, registra notas de su materia y ve el promedio calculado correctamente.</t>
   </si>
   <si>
-    <t xml:space="preserve">Días 1–2: revisión e inspección Fagan del SRS con el cliente; tabla de casos de prueba del cálculo según la RM 001/2026, firmada por el cliente (R02); inspección Fagan del SAD · Día 2: repositorio con develop y main protegidas, Husky y Jenkins Multibranch (ESLint + Prettier, Jest + cobertura, SonarQube Cloud, npm audit) · Día 5: auditoría de cierre del Sprint 1</t>
+    <t xml:space="preserve">Días 1–2: revisión e inspección Fagan del SRS con el cliente; tabla de casos de prueba del cálculo según la RM 001/2026, firmada por el cliente (R02); inspección Fagan del SAD · Día 2: repositorio con develop y main protegidas, Husky y Jenkins Multibranch; staging con despliegue continuo y smoke test (ADR-0009) (ESLint + Prettier, Jest + cobertura, SonarQube Cloud, npm audit) · Día 5: auditoría de cierre del Sprint 1</t>
   </si>
   <si>
     <t xml:space="preserve">US-04, US-03, US-19, US-05, US-10</t>
@@ -386,7 +386,7 @@
     <t xml:space="preserve">Semana 2. Las notas se corrigen con auditoría, se importan desde Excel y se registra la asistencia.</t>
   </si>
   <si>
-    <t xml:space="preserve">Día 1: revisión de diseño detallado de US-04 y US-05 · Staging con despliegue automático y smoke test · Primeros escenarios E2E de Cypress (Registrar calificación) · Día 5: auditoría de cierre del Sprint 2</t>
+    <t xml:space="preserve">Día 1: revisión de diseño detallado de US-04 y US-05 · Primeros escenarios E2E de Cypress (Registrar calificación) · Día 5: auditoría de cierre del Sprint 2</t>
   </si>
   <si>
     <t xml:space="preserve">US-06, US-07, US-20, US-11</t>
@@ -728,7 +728,7 @@
     <t xml:space="preserve">T-028</t>
   </si>
   <si>
-    <t xml:space="preserve">Staging: API en Render, web en Vercel, PostgreSQL administrado; despliegue desde el Jenkinsfile (rama develop) y smoke test del commit desplegado</t>
+    <t xml:space="preserve">Staging con despliegue continuo: API y web en Render (render.yaml, ADR-0009); despliegue desde el Jenkinsfile en cada push a develop y smoke test del commit desplegado</t>
   </si>
   <si>
     <t xml:space="preserve">T-029</t>
@@ -31069,7 +31069,7 @@
       </c>
       <c r="C19" s="22" t="n">
         <f aca="false">SUMIFS('Tareas (Sprint Backlog)'!$H$5:$H$73,'Tareas (Sprint Backlog)'!$B$5:$B$73,A19,'Tareas (Sprint Backlog)'!$F$5:$F$73,"Galvan")</f>
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="D19" s="22" t="str">
         <f aca="false">IF(B19&gt;$D$16,"Sobrecarga: "&amp;TEXT(B19-$D$16,"0")&amp;" h","OK")</f>
@@ -31077,7 +31077,7 @@
       </c>
       <c r="E19" s="22" t="str">
         <f aca="false">IF(C19&gt;$D$16,"Sobrecarga: "&amp;TEXT(C19-$D$16,"0")&amp;" h","OK")</f>
-        <v>Sobrecarga: 7 h</v>
+        <v>Sobrecarga: 13 h</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31090,7 +31090,7 @@
       </c>
       <c r="C20" s="22" t="n">
         <f aca="false">SUMIFS('Tareas (Sprint Backlog)'!$H$5:$H$73,'Tareas (Sprint Backlog)'!$B$5:$B$73,A20,'Tareas (Sprint Backlog)'!$F$5:$F$73,"Galvan")</f>
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D20" s="22" t="str">
         <f aca="false">IF(B20&gt;$D$16,"Sobrecarga: "&amp;TEXT(B20-$D$16,"0")&amp;" h","OK")</f>
@@ -32091,7 +32091,7 @@
         <v>231</v>
       </c>
       <c r="B32" s="22" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="C32" s="22" t="s">
         <v>165</v>
@@ -32123,7 +32123,7 @@
         <v>233</v>
       </c>
       <c r="B33" s="22" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="C33" s="22" t="s">
         <v>165</v>

</xml_diff>

<commit_message>
docs(docs): actualizar el estado de las tareas del Sprint 1
Tareas terminadas en "En revisión" hasta que las revise el otro integrante (DoD); T-004 sigue en proceso porque
falta la firma del cliente; T-036 empieza.

Refs: T-025
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -2525,8 +2525,10 @@
       <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="8" t="s">
-        <v>14</v>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="F5" s="8" t="n">
         <v>13</v>
@@ -2574,8 +2576,10 @@
       <c r="D6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>14</v>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="F6" s="8" t="n">
         <v>13</v>
@@ -2623,8 +2627,10 @@
       <c r="D7" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="11" t="s">
-        <v>14</v>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="F7" s="11" t="n">
         <v>13</v>
@@ -2672,8 +2678,10 @@
       <c r="D8" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>14</v>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="F8" s="11" t="n">
         <v>13</v>
@@ -2721,8 +2729,10 @@
       <c r="D9" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>14</v>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="F9" s="11" t="n">
         <v>8</v>
@@ -2819,8 +2829,10 @@
       <c r="D11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="8" t="s">
-        <v>14</v>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="F11" s="8" t="n">
         <v>8</v>
@@ -31281,8 +31293,10 @@
       <c r="H6" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I6" s="22" t="s">
-        <v>152</v>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J6" s="22" t="s">
         <v>157</v>
@@ -31345,8 +31359,10 @@
       <c r="H8" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I8" s="22" t="s">
-        <v>152</v>
+      <c r="I8" s="22" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="J8" s="22" t="s">
         <v>163</v>
@@ -31377,8 +31393,10 @@
       <c r="H9" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I9" s="22" t="s">
-        <v>152</v>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J9" s="22"/>
     </row>
@@ -31407,8 +31425,10 @@
       <c r="H10" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I10" s="22" t="s">
-        <v>152</v>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J10" s="22" t="s">
         <v>169</v>
@@ -31439,8 +31459,10 @@
       <c r="H11" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="I11" s="22" t="s">
-        <v>152</v>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J11" s="22" t="s">
         <v>172</v>
@@ -31503,8 +31525,10 @@
       <c r="H13" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="22" t="s">
-        <v>152</v>
+      <c r="I13" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J13" s="22" t="s">
         <v>179</v>
@@ -31535,8 +31559,10 @@
       <c r="H14" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="I14" s="22" t="s">
-        <v>152</v>
+      <c r="I14" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J14" s="22" t="s">
         <v>182</v>
@@ -31567,8 +31593,10 @@
       <c r="H15" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I15" s="22" t="s">
-        <v>152</v>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J15" s="22" t="s">
         <v>185</v>
@@ -31599,8 +31627,10 @@
       <c r="H16" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I16" s="22" t="s">
-        <v>152</v>
+      <c r="I16" s="22" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="J16" s="22" t="s">
         <v>189</v>
@@ -31631,8 +31661,10 @@
       <c r="H17" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I17" s="22" t="s">
-        <v>152</v>
+      <c r="I17" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J17" s="22" t="s">
         <v>193</v>
@@ -31663,8 +31695,10 @@
       <c r="H18" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="I18" s="22" t="s">
-        <v>152</v>
+      <c r="I18" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J18" s="22" t="s">
         <v>196</v>
@@ -31695,8 +31729,10 @@
       <c r="H19" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="I19" s="26" t="s">
-        <v>152</v>
+      <c r="I19" s="26" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J19" s="26" t="s">
         <v>200</v>
@@ -31791,8 +31827,10 @@
       <c r="H22" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="I22" s="26" t="s">
-        <v>152</v>
+      <c r="I22" s="26" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J22" s="26" t="s">
         <v>208</v>
@@ -31823,8 +31861,10 @@
       <c r="H23" s="26" t="n">
         <v>3</v>
       </c>
-      <c r="I23" s="26" t="s">
-        <v>152</v>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J23" s="26" t="s">
         <v>211</v>
@@ -31855,8 +31895,10 @@
       <c r="H24" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="I24" s="22" t="s">
-        <v>152</v>
+      <c r="I24" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J24" s="22" t="s">
         <v>211</v>
@@ -31887,8 +31929,10 @@
       <c r="H25" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I25" s="22" t="s">
-        <v>152</v>
+      <c r="I25" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J25" s="22" t="s">
         <v>193</v>
@@ -31919,8 +31963,10 @@
       <c r="H26" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="I26" s="26" t="s">
-        <v>152</v>
+      <c r="I26" s="26" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J26" s="26" t="s">
         <v>218</v>
@@ -31951,8 +31997,10 @@
       <c r="H27" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="I27" s="22" t="s">
-        <v>152</v>
+      <c r="I27" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J27" s="22" t="s">
         <v>221</v>
@@ -32111,8 +32159,10 @@
       <c r="H32" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="I32" s="22" t="s">
-        <v>152</v>
+      <c r="I32" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J32" s="22" t="s">
         <v>169</v>
@@ -32143,8 +32193,10 @@
       <c r="H33" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I33" s="22" t="s">
-        <v>152</v>
+      <c r="I33" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J33" s="22" t="s">
         <v>193</v>
@@ -32207,8 +32259,10 @@
       <c r="H35" s="26" t="n">
         <v>5</v>
       </c>
-      <c r="I35" s="26" t="s">
-        <v>152</v>
+      <c r="I35" s="26" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J35" s="26" t="s">
         <v>240</v>
@@ -32367,8 +32421,10 @@
       <c r="H40" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I40" s="22" t="s">
-        <v>152</v>
+      <c r="I40" s="22" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="J40" s="22" t="s">
         <v>252</v>

</xml_diff>

<commit_message>
docs(docs): issues de GitHub para cada tarea y frontend del Sprint 1 a Lujan
Las 69 tareas del backlog están como issues (#1 a #69, mismo número que
la tarea), con responsable asignado, milestone por sprint y etiquetas de
área y estado. subir_issues.py los crea o los sincroniza desde el Excel
sin duplicarlos; issues-github.md tiene la tabla tarea → issue.

Como Galvan no está disponible, Lujan toma las tareas de frontend del
Sprint 1 (T-012, T-013, T-017, T-020, T-021, T-024) y Galvan pasa a ser
su revisor. T-013, T-020 y T-021 vuelven a "En proceso": hay que
rehacerlas según el diseño de las 12 pantallas.

Refs: T-012, T-013, T-017, T-020, T-021, T-024
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -31619,10 +31619,10 @@
         <v>188</v>
       </c>
       <c r="F16" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="G16" s="22" t="s">
         <v>150</v>
-      </c>
-      <c r="G16" s="22" t="s">
-        <v>151</v>
       </c>
       <c r="H16" s="22" t="n">
         <v>3</v>
@@ -31653,17 +31653,17 @@
         <v>192</v>
       </c>
       <c r="F17" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="G17" s="22" t="s">
         <v>150</v>
-      </c>
-      <c r="G17" s="22" t="s">
-        <v>151</v>
       </c>
       <c r="H17" s="22" t="n">
         <v>2</v>
       </c>
       <c r="I17" s="22" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="J17" s="22" t="s">
@@ -31789,10 +31789,10 @@
         <v>188</v>
       </c>
       <c r="F21" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="G21" s="22" t="s">
         <v>150</v>
-      </c>
-      <c r="G21" s="22" t="s">
-        <v>151</v>
       </c>
       <c r="H21" s="22" t="n">
         <v>4</v>
@@ -31889,17 +31889,17 @@
         <v>188</v>
       </c>
       <c r="F24" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="G24" s="22" t="s">
         <v>150</v>
-      </c>
-      <c r="G24" s="22" t="s">
-        <v>151</v>
       </c>
       <c r="H24" s="22" t="n">
         <v>4</v>
       </c>
       <c r="I24" s="22" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="J24" s="22" t="s">
@@ -31923,17 +31923,17 @@
         <v>192</v>
       </c>
       <c r="F25" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="G25" s="22" t="s">
         <v>150</v>
-      </c>
-      <c r="G25" s="22" t="s">
-        <v>151</v>
       </c>
       <c r="H25" s="22" t="n">
         <v>2</v>
       </c>
       <c r="I25" s="22" t="inlineStr">
         <is>
-          <t>En revisión</t>
+          <t>En proceso</t>
         </is>
       </c>
       <c r="J25" s="22" t="s">
@@ -32025,10 +32025,10 @@
         <v>188</v>
       </c>
       <c r="F28" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="G28" s="22" t="s">
         <v>150</v>
-      </c>
-      <c r="G28" s="22" t="s">
-        <v>151</v>
       </c>
       <c r="H28" s="22" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
docs(docs): SAD con la estructura de la web y tareas de frontend en revisión
SAD 1.2 (Markdown, Word y PDF): web/src por rol, componentes, sesión,
institución y tema. Backlog: T-012, T-013, T-017, T-020, T-021 y T-024
pasan a "En revisión" (las revisa Galvan).

Refs: T-012, T-013, T-017, T-020, T-021, T-024
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -31629,7 +31629,7 @@
       </c>
       <c r="I16" s="22" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="J16" s="22" t="s">
@@ -31663,7 +31663,7 @@
       </c>
       <c r="I17" s="22" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="J17" s="22" t="s">
@@ -31797,8 +31797,10 @@
       <c r="H21" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="I21" s="22" t="s">
-        <v>152</v>
+      <c r="I21" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J21" s="22" t="s">
         <v>18</v>
@@ -31899,7 +31901,7 @@
       </c>
       <c r="I24" s="22" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="J24" s="22" t="s">
@@ -31933,7 +31935,7 @@
       </c>
       <c r="I25" s="22" t="inlineStr">
         <is>
-          <t>En proceso</t>
+          <t>En revisión</t>
         </is>
       </c>
       <c r="J25" s="22" t="s">
@@ -32033,8 +32035,10 @@
       <c r="H28" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="I28" s="22" t="s">
-        <v>152</v>
+      <c r="I28" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J28" s="22" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
feat(calculo): historial académico del estudiante por trimestre
GET /api/estudiantes/:id/historial devuelve cada trimestre de la gestión con la
nota de cada materia del curso (calculada al consultar con CalculoService), el
promedio del trimestre, el promedio anual, la tendencia y el estado. El profesor
solo ve a los estudiantes de un curso en el que dicta al menos una materia
(403 en otro caso); la secretaria y el administrador ven todos.

Decisión D12 en reglas-ministerio.md (y en el generador del backlog). T-034 en
revisión en el Excel y en issues-github.md.

Refs: US-03, T-034
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -2780,8 +2780,10 @@
       <c r="D10" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="11" t="s">
-        <v>14</v>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="F10" s="11" t="n">
         <v>10</v>
@@ -32363,8 +32365,10 @@
       <c r="H38" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I38" s="22" t="s">
-        <v>152</v>
+      <c r="I38" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J38" s="22" t="s">
         <v>247</v>

</xml_diff>

<commit_message>
feat(notas): API del control de entrega de notas por curso
La pantalla de la secretaria y el botón del profesor ya llamaban a /api/entregas,
pero la ruta no existía. Ahora:
- GET /api/entregas (secretaria, administrador): cada materia de la gestión con
  su profesor, su estado Entregado o Pendiente y los conteos de notas.
- GET /api/entregas/materias/:id: estado de una materia en un trimestre.
- POST /api/entregas/materias/:id/entregar (profesor asignado): solo si todos los
  estudiantes tienen nota en todas las actividades (criterio 2).
Tabla entregas_notas con una fila por materia y trimestre (migración nueva).
Decisión D13 en reglas-ministerio.md; rutas en la matriz M09.

Refs: US-10, T-040
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -2931,8 +2931,10 @@
       <c r="D13" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>14</v>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>En proceso</t>
+        </is>
       </c>
       <c r="F13" s="11" t="n">
         <v>5</v>
@@ -32561,8 +32563,10 @@
       <c r="H44" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="I44" s="22" t="s">
-        <v>152</v>
+      <c r="I44" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J44" s="22" t="s">
         <v>263</v>

</xml_diff>

<commit_message>
docs(docs): tareas de frontend del Sprint 2 en revisión
T-032, T-033, T-035 y T-037 funcionan contra la API y sus escenarios Cypress
pasan (21 de 21 en local).

Refs: T-032, T-033, T-035, T-037
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -32305,8 +32305,10 @@
       <c r="H36" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I36" s="22" t="s">
-        <v>152</v>
+      <c r="I36" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J36" s="22" t="s">
         <v>30</v>
@@ -32337,8 +32339,10 @@
       <c r="H37" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="I37" s="22" t="s">
-        <v>152</v>
+      <c r="I37" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J37" s="22" t="s">
         <v>193</v>
@@ -32403,8 +32407,10 @@
       <c r="H39" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I39" s="22" t="s">
-        <v>152</v>
+      <c r="I39" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J39" s="22" t="s">
         <v>35</v>
@@ -32469,8 +32475,10 @@
       <c r="H41" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="I41" s="22" t="s">
-        <v>152</v>
+      <c r="I41" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J41" s="22" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
docs(sqap): informe de pruebas y actas del Sprint 2 con lo que pasó de verdad
El informe y las actas que Galvan dejó el 20/10 daban por hechas la demo con el
cliente y las auditorías T-041 y T-042 (con la firma de Lujan) y declaraban M02
al 100 %, pero la web no compilaba y 3 archivos Cypress no podían pasar.
- informe-pruebas-sprint2.md y los JUnit rehechos con la ejecución del
  21/10 (API 214, web 123, Cypress 22; build 25 de Jenkins en verde).
- T-042: auditoría real, con hallazgos mayores (ya corregidos) y la limitación
  de independencia.
- T-041 y la revisión con el cliente quedan preparadas y pendientes: no hay
  auditor independiente y la demo no se realizó.

Refs: T-041, T-042
</commit_message>
<xml_diff>
--- a/docs/backlog/backlog_v2_4sprints.xlsx
+++ b/docs/backlog/backlog_v2_4sprints.xlsx
@@ -32643,8 +32643,10 @@
       <c r="H46" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="I46" s="22" t="s">
-        <v>152</v>
+      <c r="I46" s="22" t="inlineStr">
+        <is>
+          <t>En revisión</t>
+        </is>
       </c>
       <c r="J46" s="22" t="s">
         <v>153</v>

</xml_diff>